<commit_message>
fix(positions): ship bulk template with headers only
La plantilla incluia una fila de ejemplo (ana.perez@example.com) que el parser trata como fila de datos, por lo que descargar y subir la plantilla sin editar creaba un candidato ficticio. Ahora solo lleva la cabecera y el backend responde EXCEL_BULK_NO_ROWS si se sube vacia.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/templates/Plantilla_Carga_Masiva.xlsx
+++ b/public/templates/Plantilla_Carga_Masiva.xlsx
@@ -52,7 +52,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -101,43 +101,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ana</t>
-        </is>
-      </c>
-      <c r="B2" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Perez</t>
-        </is>
-      </c>
-      <c r="C2" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lopez</t>
-        </is>
-      </c>
-      <c r="D2" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ana.perez@example.com</t>
-        </is>
-      </c>
-      <c r="E2" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">+52</t>
-        </is>
-      </c>
-      <c r="F2" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">5512345678</t>
-        </is>
-      </c>
-      <c r="G2" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">F</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(positions): ship bulk template with headers only (#319)
fix(positions): ship bulk upload template with headers only

Plantilla sin fila de ejemplo para evitar candidato ficticio al subirla sin editar.
</commit_message>
<xml_diff>
--- a/public/templates/Plantilla_Carga_Masiva.xlsx
+++ b/public/templates/Plantilla_Carga_Masiva.xlsx
@@ -52,7 +52,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -101,43 +101,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ana</t>
-        </is>
-      </c>
-      <c r="B2" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Perez</t>
-        </is>
-      </c>
-      <c r="C2" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lopez</t>
-        </is>
-      </c>
-      <c r="D2" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ana.perez@example.com</t>
-        </is>
-      </c>
-      <c r="E2" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">+52</t>
-        </is>
-      </c>
-      <c r="F2" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">5512345678</t>
-        </is>
-      </c>
-      <c r="G2" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">F</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>